<commit_message>
Daily recap, matchup updates, learning and research 2026-08-14
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-14.xlsx
+++ b/data/k-props/2026-08-14.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="92">
   <si>
     <t>date</t>
   </si>
@@ -145,6 +145,9 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -154,12 +157,18 @@
     <t>Clay Holmes</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
     <t>Sandy Alcantara</t>
   </si>
   <si>
     <t>Miami Marlins @ Cincinnati Reds</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>&gt;=7</t>
   </si>
   <si>
@@ -200,6 +209,9 @@
   </si>
   <si>
     <t>Gavin Williams</t>
+  </si>
+  <si>
+    <t>W</t>
   </si>
   <si>
     <t>Chris Bassitt</t>
@@ -856,17 +868,23 @@
       <c r="Y2">
         <v>0.975</v>
       </c>
+      <c r="Z2">
+        <v>6</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>0.63</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>5.13</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.2368</v>
@@ -876,6 +894,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>0.87</v>
+      </c>
+      <c r="AJ2">
+        <v>0.87</v>
+      </c>
+      <c r="AK2">
+        <v>0.87</v>
+      </c>
+      <c r="AL2">
+        <v>0.87</v>
       </c>
       <c r="AM2">
         <v>5.13</v>
@@ -886,7 +916,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>3.5</v>
@@ -957,17 +987,23 @@
       <c r="Y3">
         <v>0.9708</v>
       </c>
+      <c r="Z3">
+        <v>3</v>
+      </c>
       <c r="AA3" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB3">
+        <v>0.34</v>
       </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD3">
         <v>3.84</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.1995</v>
@@ -977,6 +1013,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-0.84</v>
+      </c>
+      <c r="AJ3">
+        <v>0.84</v>
+      </c>
+      <c r="AK3">
+        <v>-0.84</v>
+      </c>
+      <c r="AL3">
+        <v>0.84</v>
       </c>
       <c r="AM3">
         <v>3.84</v>
@@ -987,7 +1035,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>5.5</v>
@@ -999,7 +1047,7 @@
         <v>102</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>824479</v>
@@ -1058,17 +1106,23 @@
       <c r="Y4">
         <v>1.062</v>
       </c>
+      <c r="Z4">
+        <v>2</v>
+      </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB4">
+        <v>1.92</v>
       </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD4">
         <v>8.22</v>
       </c>
       <c r="AE4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="AF4">
         <v>0.1993</v>
@@ -1078,6 +1132,18 @@
       </c>
       <c r="AH4">
         <v>-0.8</v>
+      </c>
+      <c r="AI4">
+        <v>-6.22</v>
+      </c>
+      <c r="AJ4">
+        <v>6.22</v>
+      </c>
+      <c r="AK4">
+        <v>-5.42</v>
+      </c>
+      <c r="AL4">
+        <v>5.42</v>
       </c>
       <c r="AM4">
         <v>7.42</v>
@@ -1088,7 +1154,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C5">
         <v>6.5</v>
@@ -1100,7 +1166,7 @@
         <v>-115</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <v>824479</v>
@@ -1159,17 +1225,23 @@
       <c r="Y5">
         <v>0.8833</v>
       </c>
+      <c r="Z5">
+        <v>8</v>
+      </c>
       <c r="AA5" t="s">
         <v>44</v>
       </c>
+      <c r="AB5">
+        <v>-0.49</v>
+      </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD5">
         <v>6.01</v>
       </c>
       <c r="AE5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="AF5">
         <v>0.2691</v>
@@ -1179,6 +1251,18 @@
       </c>
       <c r="AH5">
         <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>1.99</v>
+      </c>
+      <c r="AJ5">
+        <v>1.99</v>
+      </c>
+      <c r="AK5">
+        <v>1.99</v>
+      </c>
+      <c r="AL5">
+        <v>1.99</v>
       </c>
       <c r="AM5">
         <v>6.01</v>
@@ -1189,7 +1273,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C6">
         <v>4.5</v>
@@ -1201,7 +1285,7 @@
         <v>-146</v>
       </c>
       <c r="F6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G6">
         <v>823346</v>
@@ -1260,17 +1344,23 @@
       <c r="Y6">
         <v>1.0839</v>
       </c>
+      <c r="Z6">
+        <v>6</v>
+      </c>
       <c r="AA6" t="s">
         <v>44</v>
       </c>
+      <c r="AB6">
+        <v>0.54</v>
+      </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD6">
         <v>5.04</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
         <v>0.1736</v>
@@ -1280,6 +1370,18 @@
       </c>
       <c r="AH6">
         <v>0</v>
+      </c>
+      <c r="AI6">
+        <v>0.96</v>
+      </c>
+      <c r="AJ6">
+        <v>0.96</v>
+      </c>
+      <c r="AK6">
+        <v>0.96</v>
+      </c>
+      <c r="AL6">
+        <v>0.96</v>
       </c>
       <c r="AM6">
         <v>5.04</v>
@@ -1290,7 +1392,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C7">
         <v>4.5</v>
@@ -1302,7 +1404,7 @@
         <v>-146</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G7">
         <v>823346</v>
@@ -1361,17 +1463,23 @@
       <c r="Y7">
         <v>0.9909</v>
       </c>
+      <c r="Z7">
+        <v>5</v>
+      </c>
       <c r="AA7" t="s">
         <v>44</v>
       </c>
+      <c r="AB7">
+        <v>-0.66</v>
+      </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD7">
         <v>3.84</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
         <v>0.2096</v>
@@ -1381,6 +1489,18 @@
       </c>
       <c r="AH7">
         <v>0</v>
+      </c>
+      <c r="AI7">
+        <v>1.16</v>
+      </c>
+      <c r="AJ7">
+        <v>1.16</v>
+      </c>
+      <c r="AK7">
+        <v>1.16</v>
+      </c>
+      <c r="AL7">
+        <v>1.16</v>
       </c>
       <c r="AM7">
         <v>3.84</v>
@@ -1391,16 +1511,16 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G8">
         <v>824237</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I8">
         <v>3</v>
@@ -1454,16 +1574,16 @@
         <v>0.88</v>
       </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD8">
         <v>2.36</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.2375</v>
@@ -1483,10 +1603,10 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G9">
         <v>823591</v>
@@ -1546,16 +1666,16 @@
         <v>0.9762</v>
       </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD9">
         <v>4.12</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.1953</v>
@@ -1575,7 +1695,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C10">
         <v>3.5</v>
@@ -1587,7 +1707,7 @@
         <v>132</v>
       </c>
       <c r="F10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G10">
         <v>824399</v>
@@ -1646,17 +1766,23 @@
       <c r="Y10">
         <v>0.88</v>
       </c>
+      <c r="Z10">
+        <v>4</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD10">
         <v>3.5</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.2245</v>
@@ -1666,6 +1792,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>0.5</v>
+      </c>
+      <c r="AJ10">
+        <v>0.5</v>
+      </c>
+      <c r="AK10">
+        <v>0.5</v>
+      </c>
+      <c r="AL10">
+        <v>0.5</v>
       </c>
       <c r="AM10">
         <v>3.5</v>
@@ -1676,7 +1814,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C11">
         <v>7.5</v>
@@ -1688,7 +1826,7 @@
         <v>-155</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G11">
         <v>824399</v>
@@ -1747,17 +1885,23 @@
       <c r="Y11">
         <v>0.9878</v>
       </c>
+      <c r="Z11">
+        <v>5</v>
+      </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB11">
+        <v>-0.73</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="AD11">
         <v>6.77</v>
       </c>
       <c r="AE11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="AF11">
         <v>0.3692</v>
@@ -1767,6 +1911,18 @@
       </c>
       <c r="AH11">
         <v>0</v>
+      </c>
+      <c r="AI11">
+        <v>-1.77</v>
+      </c>
+      <c r="AJ11">
+        <v>1.77</v>
+      </c>
+      <c r="AK11">
+        <v>-1.77</v>
+      </c>
+      <c r="AL11">
+        <v>1.77</v>
       </c>
       <c r="AM11">
         <v>6.77</v>
@@ -1777,7 +1933,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>2.5</v>
@@ -1789,7 +1945,7 @@
         <v>145</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G12">
         <v>822942</v>
@@ -1848,17 +2004,23 @@
       <c r="Y12">
         <v>0.88</v>
       </c>
+      <c r="Z12">
+        <v>3</v>
+      </c>
       <c r="AA12" t="s">
         <v>44</v>
       </c>
+      <c r="AB12">
+        <v>-0.14</v>
+      </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD12">
         <v>2.36</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.1463</v>
@@ -1868,6 +2030,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>0.64</v>
+      </c>
+      <c r="AJ12">
+        <v>0.64</v>
+      </c>
+      <c r="AK12">
+        <v>0.64</v>
+      </c>
+      <c r="AL12">
+        <v>0.64</v>
       </c>
       <c r="AM12">
         <v>2.36</v>
@@ -1878,10 +2052,10 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G13">
         <v>822942</v>
@@ -1941,16 +2115,16 @@
         <v>1.0594</v>
       </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD13">
         <v>4.2</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
         <v>0.1646</v>
@@ -1970,10 +2144,10 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G14">
         <v>824882</v>
@@ -2033,16 +2207,16 @@
         <v>0.9698</v>
       </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD14">
         <v>3.05</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.1333</v>
@@ -2062,10 +2236,10 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G15">
         <v>824882</v>
@@ -2125,16 +2299,16 @@
         <v>0.88</v>
       </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD15">
         <v>5.51</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
         <v>0.3316</v>
@@ -2154,10 +2328,10 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G16">
         <v>822777</v>
@@ -2217,16 +2391,16 @@
         <v>0.9663</v>
       </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD16">
         <v>5.26</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.2885</v>
@@ -2246,10 +2420,10 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G17">
         <v>822777</v>
@@ -2309,16 +2483,16 @@
         <v>1.0349</v>
       </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD17">
         <v>4.47</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.1677</v>
@@ -2338,10 +2512,10 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G18">
         <v>824159</v>
@@ -2401,16 +2575,16 @@
         <v>1.0117</v>
       </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD18">
         <v>4.91</v>
       </c>
       <c r="AE18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF18">
         <v>0.2002</v>
@@ -2430,10 +2604,10 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G19">
         <v>824159</v>
@@ -2493,16 +2667,16 @@
         <v>0.9748</v>
       </c>
       <c r="AA19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD19">
         <v>4.56</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.2422</v>
@@ -2522,10 +2696,10 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G20">
         <v>823993</v>
@@ -2585,16 +2759,16 @@
         <v>0.9971</v>
       </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD20">
         <v>4.04</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.1688</v>
@@ -2614,10 +2788,10 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G21">
         <v>823993</v>
@@ -2677,16 +2851,16 @@
         <v>0.9424</v>
       </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD21">
         <v>3.6</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
         <v>0.2122</v>
@@ -2706,10 +2880,10 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G22">
         <v>824968</v>
@@ -2748,7 +2922,7 @@
         <v>0.373</v>
       </c>
       <c r="S22" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="T22">
         <v>0.2603</v>
@@ -2769,16 +2943,16 @@
         <v>1.013</v>
       </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD22">
         <v>5.82</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.2252</v>
@@ -2798,10 +2972,10 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F23" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G23">
         <v>823913</v>
@@ -2840,7 +3014,7 @@
         <v>0.34</v>
       </c>
       <c r="S23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="T23">
         <v>0.2813</v>
@@ -2861,16 +3035,16 @@
         <v>1.0004</v>
       </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD23">
         <v>5.99</v>
       </c>
       <c r="AE23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF23">
         <v>0.2101</v>
@@ -2890,10 +3064,10 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G24">
         <v>823913</v>
@@ -2932,7 +3106,7 @@
         <v>0.403</v>
       </c>
       <c r="S24" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="T24">
         <v>0.2018</v>
@@ -2953,16 +3127,16 @@
         <v>1.0084</v>
       </c>
       <c r="AA24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD24">
         <v>5.3</v>
       </c>
       <c r="AE24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF24">
         <v>0.2229</v>
@@ -2982,10 +3156,10 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F25" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G25">
         <v>823185</v>
@@ -3024,7 +3198,7 @@
         <v>0.396</v>
       </c>
       <c r="S25" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="T25">
         <v>0.2179</v>
@@ -3045,16 +3219,16 @@
         <v>0.9642</v>
       </c>
       <c r="AA25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD25">
         <v>4.51</v>
       </c>
       <c r="AE25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF25">
         <v>0.1925</v>
@@ -3074,10 +3248,10 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G26">
         <v>823185</v>
@@ -3137,16 +3311,16 @@
         <v>1.0107</v>
       </c>
       <c r="AA26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD26">
         <v>5.16</v>
       </c>
       <c r="AE26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF26">
         <v>0.2126</v>
@@ -3166,7 +3340,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C27">
         <v>4.5</v>
@@ -3178,31 +3352,34 @@
         <v>-101</v>
       </c>
       <c r="F27" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L27">
         <v>6</v>
       </c>
       <c r="S27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V27" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="Z27">
+        <v>4</v>
       </c>
       <c r="AA27" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>